<commit_message>
Prerequisites added to courses
</commit_message>
<xml_diff>
--- a/Back-end/Courses.xlsx
+++ b/Back-end/Courses.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Documents\SDKGU-S\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Documents\SDKGU-Subject-Sistem-new\Back-end\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EEDE0467-83AB-4A45-888E-20D4A15063AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12C5A1AD-7067-43B3-BD2D-747F330EEF2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11040" xr2:uid="{0449B7DA-74C4-4479-A92C-8080620694BE}"/>
   </bookViews>
@@ -93,9 +93,6 @@
     <t>English I: Introduction to Composition</t>
   </si>
   <si>
-    <t>ENG 202</t>
-  </si>
-  <si>
     <t>English II: Reading &amp; Writing Analytically</t>
   </si>
   <si>
@@ -105,9 +102,6 @@
     <t>Speech: Oral Communication</t>
   </si>
   <si>
-    <t>ARTS 201</t>
-  </si>
-  <si>
     <t>Introduction to Art</t>
   </si>
   <si>
@@ -448,6 +442,12 @@
   </si>
   <si>
     <t>Program ID</t>
+  </si>
+  <si>
+    <t>ENGL 202</t>
+  </si>
+  <si>
+    <t>ART 201</t>
   </si>
 </sst>
 </file>
@@ -1105,7 +1105,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="12" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="E1" s="12" t="s">
         <v>3</v>
@@ -1226,10 +1226,10 @@
     </row>
     <row r="6" spans="1:8" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>18</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>19</v>
       </c>
       <c r="C6" s="21" t="s">
         <v>9</v>
@@ -1252,10 +1252,10 @@
     </row>
     <row r="7" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>20</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>21</v>
       </c>
       <c r="C7" s="21" t="s">
         <v>9</v>
@@ -1278,10 +1278,10 @@
     </row>
     <row r="8" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>22</v>
+        <v>136</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C8" s="21" t="s">
         <v>9</v>
@@ -1304,10 +1304,10 @@
     </row>
     <row r="9" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C9" s="21" t="s">
         <v>9</v>
@@ -1330,10 +1330,10 @@
     </row>
     <row r="10" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C10" s="21" t="s">
         <v>9</v>
@@ -1356,10 +1356,10 @@
     </row>
     <row r="11" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C11" s="21" t="s">
         <v>9</v>
@@ -1382,10 +1382,10 @@
     </row>
     <row r="12" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C12" s="21" t="s">
         <v>9</v>
@@ -1408,10 +1408,10 @@
     </row>
     <row r="13" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C13" s="21" t="s">
         <v>9</v>
@@ -1434,13 +1434,13 @@
     </row>
     <row r="14" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A14" s="13" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C14" s="22" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D14" s="29">
         <v>1</v>
@@ -1460,13 +1460,13 @@
     </row>
     <row r="15" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C15" s="22" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D15" s="29">
         <v>1</v>
@@ -1486,13 +1486,13 @@
     </row>
     <row r="16" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A16" s="13" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B16" s="14" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C16" s="22" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D16" s="29">
         <v>1</v>
@@ -1512,13 +1512,13 @@
     </row>
     <row r="17" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A17" s="13" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B17" s="14" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C17" s="22" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D17" s="29">
         <v>1</v>
@@ -1538,13 +1538,13 @@
     </row>
     <row r="18" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A18" s="13" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C18" s="22" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D18" s="29">
         <v>1</v>
@@ -1564,13 +1564,13 @@
     </row>
     <row r="19" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A19" s="13" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B19" s="14" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C19" s="22" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D19" s="29">
         <v>1</v>
@@ -1590,13 +1590,13 @@
     </row>
     <row r="20" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A20" s="13" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B20" s="14" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C20" s="22" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D20" s="29">
         <v>1</v>
@@ -1616,13 +1616,13 @@
     </row>
     <row r="21" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A21" s="13" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B21" s="14" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C21" s="22" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D21" s="29">
         <v>1</v>
@@ -1642,13 +1642,13 @@
     </row>
     <row r="22" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A22" s="13" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B22" s="14" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C22" s="22" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D22" s="29">
         <v>1</v>
@@ -1668,13 +1668,13 @@
     </row>
     <row r="23" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A23" s="13" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B23" s="14" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C23" s="22" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D23" s="29">
         <v>1</v>
@@ -1694,13 +1694,13 @@
     </row>
     <row r="24" spans="1:8" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A24" s="13" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B24" s="14" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C24" s="22" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D24" s="29">
         <v>1</v>
@@ -1720,13 +1720,13 @@
     </row>
     <row r="25" spans="1:8" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A25" s="13" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B25" s="14" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C25" s="22" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D25" s="29">
         <v>1</v>
@@ -1746,13 +1746,13 @@
     </row>
     <row r="26" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A26" s="13" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B26" s="14" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C26" s="22" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D26" s="29">
         <v>1</v>
@@ -1772,13 +1772,13 @@
     </row>
     <row r="27" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A27" s="13" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B27" s="14" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C27" s="22" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D27" s="29">
         <v>1</v>
@@ -1798,13 +1798,13 @@
     </row>
     <row r="28" spans="1:8" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A28" s="13" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B28" s="14" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C28" s="22" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D28" s="29">
         <v>1</v>
@@ -1824,13 +1824,13 @@
     </row>
     <row r="29" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A29" s="13" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B29" s="14" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C29" s="22" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D29" s="29">
         <v>1</v>
@@ -1850,13 +1850,13 @@
     </row>
     <row r="30" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A30" s="13" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B30" s="14" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C30" s="22" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D30" s="29">
         <v>1</v>
@@ -1876,13 +1876,13 @@
     </row>
     <row r="31" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A31" s="13" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B31" s="14" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C31" s="22" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D31" s="29">
         <v>1</v>
@@ -1902,13 +1902,13 @@
     </row>
     <row r="32" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A32" s="13" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B32" s="14" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C32" s="22" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D32" s="29">
         <v>1</v>
@@ -1928,13 +1928,13 @@
     </row>
     <row r="33" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A33" s="13" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B33" s="14" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C33" s="22" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D33" s="29">
         <v>1</v>
@@ -1954,13 +1954,13 @@
     </row>
     <row r="34" spans="1:8" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A34" s="13" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B34" s="14" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C34" s="22" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D34" s="29">
         <v>1</v>
@@ -1980,13 +1980,13 @@
     </row>
     <row r="35" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A35" s="13" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B35" s="14" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C35" s="22" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D35" s="29">
         <v>1</v>
@@ -2006,13 +2006,13 @@
     </row>
     <row r="36" spans="1:8" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A36" s="13" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B36" s="14" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C36" s="22" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D36" s="29">
         <v>1</v>
@@ -2032,13 +2032,13 @@
     </row>
     <row r="37" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A37" s="13" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B37" s="14" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C37" s="22" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D37" s="29">
         <v>1</v>
@@ -2058,13 +2058,13 @@
     </row>
     <row r="38" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A38" s="13" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B38" s="14" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C38" s="22" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D38" s="29">
         <v>1</v>
@@ -2084,13 +2084,13 @@
     </row>
     <row r="39" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A39" s="13" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B39" s="14" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C39" s="22" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D39" s="29">
         <v>1</v>
@@ -2110,13 +2110,13 @@
     </row>
     <row r="40" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A40" s="13" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B40" s="14" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C40" s="22" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D40" s="29">
         <v>1</v>
@@ -2136,13 +2136,13 @@
     </row>
     <row r="41" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A41" s="13" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B41" s="14" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C41" s="22" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D41" s="29">
         <v>1</v>
@@ -2162,13 +2162,13 @@
     </row>
     <row r="42" spans="1:8" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A42" s="13" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B42" s="14" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C42" s="22" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D42" s="29">
         <v>1</v>
@@ -2188,13 +2188,13 @@
     </row>
     <row r="43" spans="1:8" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A43" s="13" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B43" s="19" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C43" s="22" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D43" s="29">
         <v>1</v>
@@ -2214,13 +2214,13 @@
     </row>
     <row r="44" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A44" s="7" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B44" s="7" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D44" s="27">
         <v>2</v>
@@ -2240,13 +2240,13 @@
     </row>
     <row r="45" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A45" s="7" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B45" s="20" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D45" s="27">
         <v>2</v>
@@ -2266,13 +2266,13 @@
     </row>
     <row r="46" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A46" s="7" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B46" s="20" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D46" s="27">
         <v>2</v>
@@ -2292,13 +2292,13 @@
     </row>
     <row r="47" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A47" s="7" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B47" s="20" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D47" s="27">
         <v>2</v>
@@ -2318,13 +2318,13 @@
     </row>
     <row r="48" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A48" s="7" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B48" s="20" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D48" s="27">
         <v>2</v>
@@ -2344,13 +2344,13 @@
     </row>
     <row r="49" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A49" s="7" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B49" s="20" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D49" s="27">
         <v>2</v>
@@ -2370,13 +2370,13 @@
     </row>
     <row r="50" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A50" s="7" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B50" s="20" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D50" s="27">
         <v>2</v>
@@ -2396,13 +2396,13 @@
     </row>
     <row r="51" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A51" s="7" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B51" s="20" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D51" s="27">
         <v>2</v>
@@ -2422,13 +2422,13 @@
     </row>
     <row r="52" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A52" s="7" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B52" s="20" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D52" s="27">
         <v>2</v>
@@ -2448,13 +2448,13 @@
     </row>
     <row r="53" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A53" s="7" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B53" s="20" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D53" s="27">
         <v>2</v>
@@ -2474,13 +2474,13 @@
     </row>
     <row r="54" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A54" s="7" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B54" s="20" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D54" s="27">
         <v>2</v>
@@ -2500,13 +2500,13 @@
     </row>
     <row r="55" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A55" s="7" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B55" s="20" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D55" s="27">
         <v>2</v>
@@ -2526,13 +2526,13 @@
     </row>
     <row r="56" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A56" s="7" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B56" s="20" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D56" s="27">
         <v>2</v>
@@ -2552,13 +2552,13 @@
     </row>
     <row r="57" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A57" s="7" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B57" s="20" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D57" s="27">
         <v>2</v>
@@ -2578,13 +2578,13 @@
     </row>
     <row r="58" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A58" s="7" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B58" s="20" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D58" s="27">
         <v>2</v>
@@ -2604,13 +2604,13 @@
     </row>
     <row r="59" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A59" s="7" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B59" s="20" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D59" s="27">
         <v>2</v>
@@ -2630,13 +2630,13 @@
     </row>
     <row r="60" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A60" s="7" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B60" s="20" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D60" s="27">
         <v>2</v>
@@ -2656,13 +2656,13 @@
     </row>
     <row r="61" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A61" s="7" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B61" s="20" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D61" s="27">
         <v>2</v>
@@ -2682,13 +2682,13 @@
     </row>
     <row r="62" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A62" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="B62" s="20" t="s">
+        <v>132</v>
+      </c>
+      <c r="C62" s="3" t="s">
         <v>113</v>
-      </c>
-      <c r="B62" s="20" t="s">
-        <v>134</v>
-      </c>
-      <c r="C62" s="3" t="s">
-        <v>115</v>
       </c>
       <c r="D62" s="27">
         <v>2</v>
@@ -2708,13 +2708,13 @@
     </row>
     <row r="63" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A63" s="7" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B63" s="20" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D63" s="27">
         <v>2</v>

</xml_diff>